<commit_message>
Add SOH report for 2026-10-03
</commit_message>
<xml_diff>
--- a/reports/SOH_02_10_2026.xlsx
+++ b/reports/SOH_02_10_2026.xlsx
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="E27" s="3" t="n">
         <v>40000</v>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="D57" s="2" t="n">
-        <v>602</v>
+        <v>597</v>
       </c>
       <c r="E57" s="3" t="n">
         <v>51000</v>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>1361</v>
+        <v>1356</v>
       </c>
       <c r="E59" s="3" t="n">
         <v>51000</v>
@@ -2225,7 +2225,7 @@
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="E64" s="3" t="n">
         <v>26500</v>
@@ -3957,7 +3957,7 @@
         </is>
       </c>
       <c r="D126" s="2" t="n">
-        <v>4974</v>
+        <v>4950</v>
       </c>
       <c r="E126" s="3" t="n">
         <v>2500</v>
@@ -9261,7 +9261,7 @@
         </is>
       </c>
       <c r="D319" s="2" t="n">
-        <v>651</v>
+        <v>639</v>
       </c>
       <c r="E319" s="3" t="n">
         <v>11822</v>
@@ -9289,7 +9289,7 @@
         </is>
       </c>
       <c r="D320" s="2" t="n">
-        <v>235</v>
+        <v>223</v>
       </c>
       <c r="E320" s="3" t="n">
         <v>16171</v>
@@ -14974,7 +14974,7 @@
         </is>
       </c>
       <c r="D523" s="2" t="n">
-        <v>5325</v>
+        <v>5327</v>
       </c>
       <c r="E523" s="3" t="n">
         <v>10621</v>
@@ -15534,7 +15534,7 @@
         </is>
       </c>
       <c r="D543" s="2" t="n">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="E543" s="3" t="n">
         <v>11000</v>
@@ -17551,7 +17551,7 @@
         </is>
       </c>
       <c r="D615" s="2" t="n">
-        <v>4427</v>
+        <v>4403</v>
       </c>
       <c r="E615" s="3" t="n">
         <v>10251</v>
@@ -17579,7 +17579,7 @@
         </is>
       </c>
       <c r="D616" s="2" t="n">
-        <v>500</v>
+        <v>488</v>
       </c>
       <c r="E616" s="3" t="n">
         <v>12094</v>
@@ -18559,7 +18559,7 @@
         </is>
       </c>
       <c r="D651" s="2" t="n">
-        <v>898</v>
+        <v>886</v>
       </c>
       <c r="E651" s="3" t="n">
         <v>6417</v>
@@ -22507,7 +22507,7 @@
         </is>
       </c>
       <c r="D792" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E792" s="3" t="n">
         <v>9499</v>
@@ -24132,7 +24132,7 @@
         </is>
       </c>
       <c r="D850" s="2" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E850" s="3" t="n">
         <v>8039</v>
@@ -28952,7 +28952,7 @@
         </is>
       </c>
       <c r="D1022" s="2" t="n">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="E1022" s="3" t="n">
         <v>14904</v>
@@ -29513,7 +29513,7 @@
         </is>
       </c>
       <c r="D1042" s="2" t="n">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="E1042" s="3" t="n">
         <v>7008</v>
@@ -30493,7 +30493,7 @@
         </is>
       </c>
       <c r="D1077" s="2" t="n">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="E1077" s="3" t="n">
         <v>11027</v>
@@ -35953,7 +35953,7 @@
         </is>
       </c>
       <c r="D1272" s="2" t="n">
-        <v>281</v>
+        <v>269</v>
       </c>
       <c r="E1272" s="3" t="n">
         <v>10600</v>
@@ -38333,7 +38333,7 @@
         </is>
       </c>
       <c r="D1357" s="2" t="n">
-        <v>834</v>
+        <v>822</v>
       </c>
       <c r="E1357" s="3" t="n">
         <v>10487</v>
@@ -39901,7 +39901,7 @@
         </is>
       </c>
       <c r="D1413" s="2" t="n">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="E1413" s="3" t="n">
         <v>8626</v>
@@ -40657,7 +40657,7 @@
         </is>
       </c>
       <c r="D1440" s="2" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E1440" s="3" t="n">
         <v>10733</v>
@@ -41833,7 +41833,7 @@
         </is>
       </c>
       <c r="D1482" s="2" t="n">
-        <v>236</v>
+        <v>212</v>
       </c>
       <c r="E1482" s="3" t="n">
         <v>11171</v>
@@ -43935,7 +43935,7 @@
         </is>
       </c>
       <c r="D1557" s="2" t="n">
-        <v>510</v>
+        <v>498</v>
       </c>
       <c r="E1557" s="3" t="n">
         <v>19684</v>

</xml_diff>